<commit_message>
Lab 2 Task 2 = measure a band-pass filter like Exercises 6-7 with the team's own C (10/22/47 nF) and R (100/220 Ω): submit f0 (4) and BW (5, R/(2πL), 20 %/35 %); no Q, no design, no capacitors in parallel; formulas slide removed; Excel template without fixed frequencies
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/courses/SE009/files/Lab2_RLC_data_template.xlsx
+++ b/public/courses/SE009/files/Lab2_RLC_data_template.xlsx
@@ -233,8 +233,8 @@
         <scaling>
           <logBase val="10"/>
           <orientation val="minMax"/>
-          <max val="200"/>
-          <min val="5"/>
+          <max val="250"/>
+          <min val="2"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -635,7 +635,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Filter type:</t>
+          <t>C and R (Task 2):</t>
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
@@ -663,9 +663,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n">
-        <v>8.1</v>
-      </c>
+      <c r="A6" s="4" t="n"/>
       <c r="B6" s="4" t="n"/>
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="5">
@@ -674,9 +672,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n">
-        <v>16.2</v>
-      </c>
+      <c r="A7" s="4" t="n"/>
       <c r="B7" s="4" t="n"/>
       <c r="C7" s="4" t="n"/>
       <c r="D7" s="5">
@@ -685,9 +681,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n">
-        <v>22.6</v>
-      </c>
+      <c r="A8" s="4" t="n"/>
       <c r="B8" s="4" t="n"/>
       <c r="C8" s="4" t="n"/>
       <c r="D8" s="5">
@@ -696,9 +690,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>27.5</v>
-      </c>
+      <c r="A9" s="4" t="n"/>
       <c r="B9" s="4" t="n"/>
       <c r="C9" s="4" t="n"/>
       <c r="D9" s="5">
@@ -707,9 +699,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n">
-        <v>32.4</v>
-      </c>
+      <c r="A10" s="4" t="n"/>
       <c r="B10" s="4" t="n"/>
       <c r="C10" s="4" t="n"/>
       <c r="D10" s="5">
@@ -718,9 +708,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>37.2</v>
-      </c>
+      <c r="A11" s="4" t="n"/>
       <c r="B11" s="4" t="n"/>
       <c r="C11" s="4" t="n"/>
       <c r="D11" s="5">
@@ -729,9 +717,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n">
-        <v>45.3</v>
-      </c>
+      <c r="A12" s="4" t="n"/>
       <c r="B12" s="4" t="n"/>
       <c r="C12" s="4" t="n"/>
       <c r="D12" s="5">
@@ -740,9 +726,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n">
-        <v>64.7</v>
-      </c>
+      <c r="A13" s="4" t="n"/>
       <c r="B13" s="4" t="n"/>
       <c r="C13" s="4" t="n"/>
       <c r="D13" s="5">
@@ -751,9 +735,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="n">
-        <v>129.4</v>
-      </c>
+      <c r="A14" s="4" t="n"/>
       <c r="B14" s="4" t="n"/>
       <c r="C14" s="4" t="n"/>
       <c r="D14" s="5">
@@ -863,7 +845,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rows 15–25: add extra points near the peak (any order is fine).</t>
+          <t>Rows 6–14: the 9 frequencies of your card. Rows 15–25: extra points near the peak (any order is fine).</t>
         </is>
       </c>
     </row>

</xml_diff>